<commit_message>
Updates to reserve margin and capacity retirements (to remove economic retirements of CCGTs given contract structure in Korea)
</commit_message>
<xml_diff>
--- a/InputData/elec/CRpUNL/Cap Ret per Unit Net Loss.xlsx
+++ b/InputData/elec/CRpUNL/Cap Ret per Unit Net Loss.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Dropbox\NEXT Group\90. 개인 폴더\이지우\단기대응\202501 EPS 수요전망\V3\elec\CRpUNL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\CRpUNL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A28F10E-E830-4E57-BC58-C1C329A904AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FA3AA9-EA4C-441E-BB23-CA25D856A627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4092" yWindow="1080" windowWidth="20544" windowHeight="10932" activeTab="1" xr2:uid="{67B50A2A-83E2-40E1-A966-DC033ADD8EBF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{67B50A2A-83E2-40E1-A966-DC033ADD8EBF}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -150,11 +150,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -162,7 +162,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -170,20 +170,20 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -218,7 +218,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -234,9 +234,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -274,7 +274,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -380,7 +380,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -522,7 +522,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -531,14 +531,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B7A547-DAFD-4CBC-90C6-A86A1413C282}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -546,42 +546,42 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:1">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -598,12 +598,12 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.09765625" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
@@ -611,7 +611,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -619,7 +619,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -628,16 +628,15 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4">
-        <f>$B$2</f>
-        <v>1.4999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -646,7 +645,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -654,7 +653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -663,7 +662,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -672,7 +671,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -680,7 +679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -688,7 +687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -696,7 +695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -704,7 +703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -713,7 +712,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -722,7 +721,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -731,7 +730,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -739,7 +738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -747,7 +746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -755,7 +754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -764,7 +763,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -773,7 +772,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -782,7 +781,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -791,7 +790,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -800,7 +799,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:2">
       <c r="A24" s="3" t="s">
         <v>26</v>
       </c>
@@ -809,7 +808,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:2">
       <c r="A25" s="3" t="s">
         <v>27</v>
       </c>
@@ -826,6 +825,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -969,29 +983,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{876A93A6-7E8B-49A6-A010-B55DAC4BF773}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6714B440-5469-4711-A370-119BD6291492}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B69AE32-B9EB-46AE-B3AC-403A1AED187C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6714B440-5469-4711-A370-119BD6291492}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{876A93A6-7E8B-49A6-A010-B55DAC4BF773}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B69AE32-B9EB-46AE-B3AC-403A1AED187C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated capacity retirements to calibrate korea grid size versus US
</commit_message>
<xml_diff>
--- a/InputData/elec/CRpUNL/Cap Ret per Unit Net Loss.xlsx
+++ b/InputData/elec/CRpUNL/Cap Ret per Unit Net Loss.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\CRpUNL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4FA3AA9-EA4C-441E-BB23-CA25D856A627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D98EF2E-CF4F-49E4-AC45-54157BAC6B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{67B50A2A-83E2-40E1-A966-DC033ADD8EBF}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="CRpUNL" sheetId="2" r:id="rId2"/>
+    <sheet name="US to Korea Ratio" sheetId="3" r:id="rId2"/>
+    <sheet name="CRpUNL" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t xml:space="preserve">Sources: </t>
   </si>
@@ -145,12 +146,21 @@
     <t>Certain plant types are less prone to economic retirement because they are maintained for local reliability purposes.</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
+  <si>
+    <t>US Grid</t>
+  </si>
+  <si>
+    <t>Korea Grid</t>
+  </si>
+  <si>
+    <t>Multiplier</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,6 +198,12 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -209,13 +225,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -593,6 +610,42 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EECBB9C-C9FB-4867-9A33-F95A3817E0A5}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="4">
+        <v>1324740.5</v>
+      </c>
+      <c r="B2">
+        <v>588046.50300000003</v>
+      </c>
+      <c r="C2">
+        <f>B2/A2</f>
+        <v>0.44389561804745914</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{498B6747-53CF-4C1D-84DD-4D89524F3F28}">
   <sheetPr>
     <tabColor rgb="FF002060"/>
@@ -616,7 +669,8 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>1.4999999999999999E-2</v>
+        <f>0.015*'US to Korea Ratio'!$C$2</f>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -625,7 +679,7 @@
       </c>
       <c r="B3">
         <f>$B$2</f>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -642,7 +696,7 @@
       </c>
       <c r="B5">
         <f>$B$2</f>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -659,7 +713,7 @@
       </c>
       <c r="B7">
         <f>$B$2</f>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -668,7 +722,7 @@
       </c>
       <c r="B8">
         <f>$B$2</f>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -709,7 +763,7 @@
       </c>
       <c r="B13">
         <f>$B$2</f>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -718,7 +772,7 @@
       </c>
       <c r="B14">
         <f>$B$2</f>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -727,7 +781,7 @@
       </c>
       <c r="B15">
         <f>$B$2</f>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -760,7 +814,7 @@
       </c>
       <c r="B19">
         <f t="shared" ref="B19:B25" si="0">$B$2</f>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -769,7 +823,7 @@
       </c>
       <c r="B20">
         <f t="shared" si="0"/>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -778,7 +832,7 @@
       </c>
       <c r="B21">
         <f t="shared" si="0"/>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="22" spans="1:2">
@@ -787,7 +841,7 @@
       </c>
       <c r="B22">
         <f t="shared" si="0"/>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -796,7 +850,7 @@
       </c>
       <c r="B23">
         <f t="shared" si="0"/>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -805,7 +859,7 @@
       </c>
       <c r="B24">
         <f t="shared" si="0"/>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -814,7 +868,7 @@
       </c>
       <c r="B25">
         <f t="shared" si="0"/>
-        <v>1.4999999999999999E-2</v>
+        <v>6.6584342707118865E-3</v>
       </c>
     </row>
   </sheetData>
@@ -825,21 +879,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -983,24 +1022,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{876A93A6-7E8B-49A6-A010-B55DAC4BF773}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6714B440-5469-4711-A370-119BD6291492}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B69AE32-B9EB-46AE-B3AC-403A1AED187C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1016,4 +1053,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6714B440-5469-4711-A370-119BD6291492}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{876A93A6-7E8B-49A6-A010-B55DAC4BF773}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>